<commit_message>
chore: actualización semanal 2026-03-24
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,12 +549,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>03/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — Cuenta de segundo informe de comisión .</t>
+          <t>Primer trámite constitucional / Senado — Cuenta del Mensaje 2-374 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional</t>
+          <t>Primer trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional — Comisión de Gobierno Interior (segundo informe)</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional (refundido con Bols. 16.593-06 y 16.988-06)</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Primer trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos. — Oficio</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional — Comisión de Gobierno Interior (primer informe)</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional — Comisión de Gobierno Interior (primer informe)</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional — Comisión de Gobierno Interior (primer informe)</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat: agregar columnas Urgencia, Ubicación y Comisión al seguimiento
- Nueva columna Urgencia (Col5): obtiene urgencia actual desde datos_proy del Senado
- Nueva columna Ubicación (Col6): deriva Senado/Cámara desde estado de tramitación
- Nueva columna Comisión (Col7): extrae nombre de comisión actual o "En Sala" si está en sala
- Scraping ampliado: obtiene subetapa desde datos_proy en una sola llamada adicional
- Si el nombre del proyecto está vacío, completa automáticamente título, fecha, tipo, cámara y autores
- Excel actualizado con los nuevos datos para los 11 boletines

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -60,7 +60,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -82,11 +82,17 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -108,6 +114,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -475,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -510,27 +525,42 @@
           <t>Último movimiento</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Urgencia</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>Comisión</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Fecha de presentación</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Estado de tramitación</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Tipo de iniciativa</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Cámara de origen</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Autores</t>
         </is>
@@ -557,27 +587,42 @@
           <t>Primer trámite constitucional / Senado — Cuenta del Mensaje 2-374 que hace presente la urgencia Suma</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>Suma</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>En Sala</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>10 de enero de 2024</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Mensaje</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
@@ -604,27 +649,42 @@
           <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>Gobierno, Descentralización y Regionalización</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>3 de enero de 2023</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Moción</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
@@ -651,27 +711,42 @@
           <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Suma</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>1 de septiembre de 2025</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Mensaje</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Ministerio Secretaría General de Gobierno</t>
         </is>
@@ -698,27 +773,42 @@
           <t>Primer trámite constitucional / C.Diputados — Cuenta, oficio N° 282-2025 de la Corte Suprema, por el cual remite opinión respecto del proyecto (informe N° 30-2025).</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Constitución, Legislación, Justicia y Reglamento</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>8 de septiembre de 2025</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Mensaje</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>Ministerio de Justicia y Derechos Humanos</t>
         </is>
@@ -745,27 +835,42 @@
           <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>29 de mayo de 2024</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>Moción</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
         </is>
@@ -792,27 +897,42 @@
           <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1603-373 que hace presente la urgencia Simple</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>En Sala</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>31 de mayo de 2024</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>Mensaje</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
@@ -826,7 +946,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Sin información disponible</t>
+          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -839,29 +959,44 @@
           <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>3 de abril de 2025</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Moción</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Senado</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Isabel Allende Bussi</t>
         </is>
       </c>
     </row>
@@ -873,7 +1008,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Sin información disponible</t>
+          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -886,29 +1021,44 @@
           <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Derechos Humanos y Pueblos Originarios</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>5 de mayo de 2025</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Moción</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>Cámara de Diputados</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
         </is>
       </c>
     </row>
@@ -933,27 +1083,42 @@
           <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>4 de julio de 2023</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>Moción</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
         </is>
@@ -980,27 +1145,42 @@
           <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>3 de julio de 2023</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>Moción</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
         </is>
@@ -1027,27 +1207,42 @@
           <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior, Nacionalidad, Ciudadanía y Regionalización.</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>3 de julio de 2023</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
         <is>
           <t>Moción</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
         </is>

</xml_diff>

<commit_message>
Estandarizar diseño del Excel: bordes, fill alternado y alineación uniforme
- Agrega función estandarizar_formato() que aplica diseño consistente a todas las celdas de datos
- Corrige bordes faltantes en columnas E, F, G
- Corrige fill alternado incompleto (algunas celdas dentro de una fila sin color)
- Define alineación horizontal explícita en todas las columnas (center o left según tipo)
- La función se ejecuta automáticamente al final de cada actualización semanal

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -92,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -123,6 +123,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -567,12 +573,12 @@
       </c>
     </row>
     <row r="2" ht="70" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>16.552-12</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
@@ -582,22 +588,22 @@
           <t>17/03/2026</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado — Cuenta del Mensaje 2-374 que hace presente la urgencia Suma</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Suma</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>En Sala</t>
         </is>
@@ -607,7 +613,7 @@
           <t>10 de enero de 2024</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado</t>
         </is>
@@ -622,19 +628,19 @@
           <t>Senado</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>15.643-06</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
@@ -644,22 +650,22 @@
           <t>03/10/2023</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
+      <c r="G3" s="12" t="inlineStr">
         <is>
           <t>Gobierno, Descentralización y Regionalización</t>
         </is>
@@ -669,7 +675,7 @@
           <t>3 de enero de 2023</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I3" s="12" t="inlineStr">
         <is>
           <t>Segundo trámite constitucional / Senado</t>
         </is>
@@ -684,19 +690,19 @@
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="L3" s="12" t="inlineStr">
         <is>
           <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>17.797-06</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
         </is>
@@ -706,22 +712,22 @@
           <t>02/03/2026</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Suma</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
@@ -731,7 +737,7 @@
           <t>1 de septiembre de 2025</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
@@ -746,19 +752,19 @@
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="11" t="inlineStr">
         <is>
           <t>Ministerio Secretaría General de Gobierno</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>17.817-07</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
         </is>
@@ -768,22 +774,22 @@
           <t>07/01/2026</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Cuenta, oficio N° 282-2025 de la Corte Suprema, por el cual remite opinión respecto del proyecto (informe N° 30-2025).</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>Constitución, Legislación, Justicia y Reglamento</t>
         </is>
@@ -793,7 +799,7 @@
           <t>8 de septiembre de 2025</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
@@ -808,19 +814,19 @@
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="12" t="inlineStr">
         <is>
           <t>Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>16.886-12</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Proyecto de materia medioambiental (título no indexado en fuentes públicas)</t>
         </is>
@@ -830,22 +836,22 @@
           <t>08/10/2025</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
@@ -855,7 +861,7 @@
           <t>29 de mayo de 2024</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>Segundo trámite constitucional / Senado</t>
         </is>
@@ -870,19 +876,19 @@
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L6" s="11" t="inlineStr">
         <is>
           <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>16.888-06</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
@@ -892,22 +898,22 @@
           <t>02/03/2026</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1603-373 que hace presente la urgencia Simple</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Simple</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr">
         <is>
           <t>En Sala</t>
         </is>
@@ -917,7 +923,7 @@
           <t>31 de mayo de 2024</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I7" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
@@ -932,19 +938,19 @@
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L7" s="6" t="inlineStr">
+      <c r="L7" s="12" t="inlineStr">
         <is>
           <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>17.446-17</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
         </is>
@@ -954,32 +960,32 @@
           <t>08/04/2025</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>3 de abril de 2025</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / Senado</t>
         </is>
@@ -994,19 +1000,19 @@
           <t>Senado</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="L8" s="11" t="inlineStr">
         <is>
           <t>Isabel Allende Bussi</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>17.520-17</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
         </is>
@@ -1016,32 +1022,32 @@
           <t>07/05/2025</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>Derechos Humanos y Pueblos Originarios</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>5 de mayo de 2025</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I9" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
@@ -1056,19 +1062,19 @@
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="L9" s="12" t="inlineStr">
         <is>
           <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
         </is>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>16.075-06</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
         </is>
@@ -1078,22 +1084,22 @@
           <t>11/07/2023</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
@@ -1103,7 +1109,7 @@
           <t>4 de julio de 2023</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
@@ -1118,19 +1124,19 @@
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="L10" s="11" t="inlineStr">
         <is>
           <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
         </is>
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>16.064-06</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
         </is>
@@ -1140,22 +1146,22 @@
           <t>05/07/2023</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
@@ -1165,7 +1171,7 @@
           <t>3 de julio de 2023</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
@@ -1180,19 +1186,19 @@
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
+      <c r="L11" s="12" t="inlineStr">
         <is>
           <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
         </is>
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>16.063-06</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
         </is>
@@ -1202,22 +1208,22 @@
           <t>05/07/2023</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior, Nacionalidad, Ciudadanía y Regionalización.</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
@@ -1227,7 +1233,7 @@
           <t>3 de julio de 2023</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
@@ -1242,7 +1248,7 @@
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="L12" s="11" t="inlineStr">
         <is>
           <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
         </is>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-03-27
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -595,7 +595,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-04-13
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,17 +585,17 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — Cuenta del Mensaje 2-374 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / Senado — Discusión particular . Queda pendiente</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Discusión inmediata</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / Senado — DiarioVotación</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -647,17 +647,17 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>03/10/2023</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Gobierno, Descentralización y Regionalización</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 27-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Corrige nombre del boletín 16.886-12 y mejora detección de títulos genéricos
- Actualiza nombre del boletín 16.886-12 en el Excel con el título real del Senado
- Script ahora re-consulta la API cuando el nombre contiene "no indexado"

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -828,7 +828,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Proyecto de materia medioambiental (título no indexado en fuentes públicas)</t>
+          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Corrige nombre del boletín 16.886-12 en Excel
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -828,7 +828,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Proyecto de materia medioambiental (título no indexado en fuentes públicas)</t>
+          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-04-14
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Agrega boletín 16746-06 al seguimiento
Ley N° 20.285 (transparencia empresas públicas) — Primer trámite C.Diputados, urgencia Simple.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1251,6 +1251,68 @@
       <c r="L12" s="11" t="inlineStr">
         <is>
           <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>16746-06</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>23/03/2026</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Miércoles 10 de Abril, 2024</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / C.Diputados</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>Moción</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>C.Diputados</t>
+        </is>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-04-20
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — Discusión particular . Queda pendiente</t>
+          <t>Primer trámite constitucional / Senado — Discusión particular . Aprobado</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Cuenta de proyecto</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-04-24
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,27 +585,27 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — Discusión particular . Aprobado</t>
+          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 47-374 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Discusión inmediata</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Cuenta de proyecto</t>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — DiarioVotación</t>
+          <t>Segundo trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Agrega boletín 18216-05, hipervínculos en Excel y correo
- Nuevo boletín 18216-05 (Reconstrucción nacional, urgencia Suma)
- Hipervínculos en columna boletín del Excel (www.senado.cl boletin_ini=)
- Hipervínculos preservados al reordenar filas (_aplicar_hyperlinks)
- Links a boletines en las tres secciones del correo HTML
- Excel ordenado por fecha de último movimiento

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -573,24 +573,24 @@
       </c>
     </row>
     <row r="2" ht="70" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>16.552-12</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 47-374 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 62-374 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -605,17 +605,17 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>Hacienda</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>Miércoles 22 de Abril, 2026</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -625,39 +625,39 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Hacienda</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>15.643-06</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 27-374 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / Senado — Discusión particular . Queda pendiente</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Discusión inmediata</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -667,54 +667,54 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>3 de enero de 2023</t>
+          <t>10 de enero de 2024</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / Senado — DiarioVotación</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>16746-06</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 27-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -724,22 +724,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Abril, 2024</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -749,39 +749,39 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>17.797-06</t>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>16746-06</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
+          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>1 de septiembre de 2025</t>
+          <t>Miércoles 10 de Abril, 2024</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
@@ -806,29 +806,29 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno</t>
+          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>16.888-06</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>17.797-06</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
+          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -838,12 +838,12 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1603-373 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -853,12 +853,12 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>31 de mayo de 2024</t>
+          <t>1 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -878,34 +878,34 @@
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
+          <t>Ministerio Secretaría General de Gobierno</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>17.817-07</t>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>16.888-06</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
+          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>07/01/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta, oficio N° 282-2025 de la Corte Suprema, por el cual remite opinión respecto del proyecto (informe N° 30-2025).</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1603-373 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Constitución, Legislación, Justicia y Reglamento</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>8 de septiembre de 2025</t>
+          <t>31 de mayo de 2024</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
@@ -940,29 +940,29 @@
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Justicia y Derechos Humanos</t>
+          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>16.886-12</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>17.817-07</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
+          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>07/01/2026</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta, oficio N° 282-2025 de la Corte Suprema, por el cual remite opinión respecto del proyecto (informe N° 30-2025).</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -972,27 +972,27 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Constitución, Legislación, Justicia y Reglamento</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>29 de mayo de 2024</t>
+          <t>8 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -1002,29 +1002,29 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
+          <t>Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>17.520-17</t>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>16.886-12</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
+          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>07/05/2025</t>
+          <t>08/10/2025</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1034,22 +1034,22 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Derechos Humanos y Pueblos Originarios</t>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>5 de mayo de 2025</t>
+          <t>29 de mayo de 2024</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
@@ -1064,29 +1064,29 @@
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
+          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
         </is>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>17.446-17</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>17.520-17</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
+          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1096,22 +1096,22 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Derechos Humanos y Pueblos Originarios</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>3 de abril de 2025</t>
+          <t>5 de mayo de 2025</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1121,34 +1121,34 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>Isabel Allende Bussi</t>
+          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
         </is>
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>16.075-06</t>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>17.446-17</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
+          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>11/07/2023</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1158,22 +1158,22 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>4 de julio de 2023</t>
+          <t>3 de abril de 2025</t>
         </is>
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -1183,29 +1183,29 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
+          <t>Isabel Allende Bussi</t>
         </is>
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>16.064-06</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>16.075-06</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
+          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>05/07/2023</t>
+          <t>11/07/2023</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>3 de julio de 2023</t>
+          <t>4 de julio de 2023</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -1250,67 +1250,129 @@
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
+          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>16.064-06</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>05/07/2023</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>3 de julio de 2023</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / C.Diputados</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>Moción</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>Cámara de Diputados</t>
+        </is>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>16.063-06</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>05/07/2023</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior, Nacionalidad, Ciudadanía y Regionalización.</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>3 de julio de 2023</t>
         </is>
       </c>
-      <c r="I13" s="12" t="inlineStr">
+      <c r="I14" s="11" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Moción</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L13" s="12" t="inlineStr">
+      <c r="L14" s="11" t="inlineStr">
         <is>
           <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
         </is>
@@ -1329,6 +1391,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-04-27
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 62-374 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio N° 21184. Oficio a la Corte Suprema.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-05-04
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -575,27 +575,27 @@
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>18216-05</t>
+          <t>16.888-06</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
+          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio N° 21184. Oficio a la Corte Suprema.</t>
+          <t>Primer trámite constitucional / C.Diputados — Primer informe de comisión de Hacienda.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -605,17 +605,17 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Hacienda</t>
+          <t>Cuenta de primer informe de comisión</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 22 de Abril, 2026</t>
+          <t>31 de mayo de 2024</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -625,34 +625,34 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Hacienda</t>
+          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 47-374 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio N° 21184. Oficio a la Corte Suprema.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -667,17 +667,17 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>Hacienda</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>Miércoles 22 de Abril, 2026</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -687,96 +687,96 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Hacienda</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>15.643-06</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 27-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 47-374 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>10 de enero de 2024</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Segundo trámite constitucional / C.Diputados</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Mensaje</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>3 de enero de 2023</t>
-        </is>
-      </c>
-      <c r="I4" s="11" t="inlineStr">
-        <is>
-          <t>Segundo trámite constitucional / Senado</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Moción</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Cámara de Diputados</t>
-        </is>
-      </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>16746-06</t>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 27-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -786,22 +786,22 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Abril, 2024</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -811,39 +811,39 @@
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>17.797-06</t>
+          <t>16746-06</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
+          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>1 de septiembre de 2025</t>
+          <t>Miércoles 10 de Abril, 2024</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -868,29 +868,29 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno</t>
+          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>16.888-06</t>
+          <t>17.797-06</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
+          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1603-373 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>31 de mayo de 2024</t>
+          <t>1 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
+          <t>Ministerio Secretaría General de Gobierno</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-05-11
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -575,27 +575,27 @@
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>16.888-06</t>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Primer informe de comisión de Hacienda.</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 78-374 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -605,12 +605,12 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Cuenta de primer informe de comisión</t>
+          <t>Hacienda</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>31 de mayo de 2024</t>
+          <t>Miércoles 22 de Abril, 2026</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
@@ -625,101 +625,101 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
+          <t>Ministerio de Hacienda</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>18216-05</t>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio N° 21184. Oficio a la Corte Suprema.</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 76-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Hacienda</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Miércoles 22 de Abril, 2026</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Hacienda</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>16.888-06</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 47-374 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta de primer informe de comisión .</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -729,17 +729,17 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>31 de mayo de 2024</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -749,34 +749,34 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>15.643-06</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 27-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 69-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -786,37 +786,37 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>10 de enero de 2024</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>Segundo trámite constitucional / C.Diputados</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Mensaje</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>3 de enero de 2023</t>
-        </is>
-      </c>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>Segundo trámite constitucional / Senado</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Moción</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>Cámara de Diputados</t>
-        </is>
-      </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-05-12
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 78-374 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta oficio N? 116-2026 de la Corte Suprema</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-05-18
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta oficio N? 116-2026 de la Corte Suprema</t>
+          <t>Primer trámite constitucional / C.Diputados — S.E. el Presidente de la República formula indicaciones al proyecto. (037-374). Incluye informe financiero complementario N° 097/13.05.2026.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -637,22 +637,22 @@
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>15.643-06</t>
+          <t>16.888-06</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 76-374 que retira y hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -662,27 +662,27 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>3 de enero de 2023</t>
+          <t>31 de mayo de 2024</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados — Diario</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -692,29 +692,29 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16.888-06</t>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta de primer informe de comisión .</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 76-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -724,27 +724,27 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>31 de mayo de 2024</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-05-25
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — S.E. el Presidente de la República formula indicaciones al proyecto. (037-374). Incluye informe financiero complementario N° 097/13.05.2026.</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del informe de la Comisión de Hacienda, del de la Comisión de Medio Ambiente, y del certificado de la Comisión de Trabajo</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Agrega boletín 16553-12 al seguimiento
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -699,27 +699,27 @@
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>15.643-06</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 76-374 que retira y hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Segundo informe de comisión de Medio Ambiente, Cambio Climático y Bienes Nacionales.  COMPARADO DE INDICACIONES</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -729,54 +729,54 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>3 de enero de 2023</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Segundo trámite constitucional / Senado — Comparado</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 69-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 76-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -786,59 +786,59 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>16746-06</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 69-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -853,59 +853,59 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Abril, 2024</t>
+          <t>10 de enero de 2024</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>17.797-06</t>
+          <t>16746-06</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
+          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>1 de septiembre de 2025</t>
+          <t>Miércoles 10 de Abril, 2024</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
@@ -930,44 +930,44 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno</t>
+          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>17.817-07</t>
+          <t>17.797-06</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
+          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>07/01/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta, oficio N° 282-2025 de la Corte Suprema, por el cual remite opinión respecto del proyecto (informe N° 30-2025).</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Constitución, Legislación, Justicia y Reglamento</t>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>8 de septiembre de 2025</t>
+          <t>1 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -1002,29 +1002,29 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Justicia y Derechos Humanos</t>
+          <t>Ministerio Secretaría General de Gobierno</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>16.886-12</t>
+          <t>17.817-07</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
+          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>07/01/2026</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta, oficio N° 282-2025 de la Corte Suprema, por el cual remite opinión respecto del proyecto (informe N° 30-2025).</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1034,27 +1034,27 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Constitución, Legislación, Justicia y Reglamento</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>29 de mayo de 2024</t>
+          <t>8 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1064,29 +1064,29 @@
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
+          <t>Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>17.520-17</t>
+          <t>16.886-12</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
+          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>07/05/2025</t>
+          <t>08/10/2025</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1096,22 +1096,22 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Derechos Humanos y Pueblos Originarios</t>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>5 de mayo de 2025</t>
+          <t>29 de mayo de 2024</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1126,29 +1126,29 @@
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
+          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
         </is>
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>17.446-17</t>
+          <t>17.520-17</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
+          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1158,22 +1158,22 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Derechos Humanos y Pueblos Originarios</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>3 de abril de 2025</t>
+          <t>5 de mayo de 2025</t>
         </is>
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -1183,34 +1183,34 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>Isabel Allende Bussi</t>
+          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
         </is>
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>16.075-06</t>
+          <t>17.446-17</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
+          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>11/07/2023</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1220,22 +1220,22 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>4 de julio de 2023</t>
+          <t>3 de abril de 2025</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1245,29 +1245,29 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
+          <t>Isabel Allende Bussi</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>16.064-06</t>
+          <t>16.075-06</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
+          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>05/07/2023</t>
+          <t>11/07/2023</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>3 de julio de 2023</t>
+          <t>4 de julio de 2023</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
@@ -1312,67 +1312,129 @@
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
+          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>16.064-06</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>05/07/2023</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Sin urgencia</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>3 de julio de 2023</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Primer trámite constitucional / C.Diputados</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Moción</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Cámara de Diputados</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="inlineStr">
+        <is>
+          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t>16.063-06</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>05/07/2023</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior, Nacionalidad, Ciudadanía y Regionalización.</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>Sin urgencia</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="G14" s="11" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>3 de julio de 2023</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr">
+      <c r="I15" s="12" t="inlineStr">
         <is>
           <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J15" s="7" t="inlineStr">
         <is>
           <t>Moción</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K15" s="7" t="inlineStr">
         <is>
           <t>Cámara de Diputados</t>
         </is>
       </c>
-      <c r="L14" s="11" t="inlineStr">
+      <c r="L15" s="12" t="inlineStr">
         <is>
           <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
         </is>
@@ -1393,6 +1455,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-05-27
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Seguimiento Legislativo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del informe de la Comisión de Hacienda, del de la Comisión de Medio Ambiente, y del certificado de la Comisión de Trabajo</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio de ley a Cámara Revisora .</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Hacienda</t>
+          <t>Cuenta de proyecto</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-06-08
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio de ley a Cámara Revisora .</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 111-374 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -600,12 +600,12 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Cuenta de proyecto</t>
+          <t>Hacienda</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -637,22 +637,22 @@
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>16.888-06</t>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 123-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -662,27 +662,27 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>31 de mayo de 2024</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Diario</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -692,91 +692,91 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Segundo informe de comisión de Medio Ambiente, Cambio Climático y Bienes Nacionales.  COMPARADO DE INDICACIONES</t>
+          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 121-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>10 de enero de 2024</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Segundo trámite constitucional / C.Diputados</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Mensaje</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Miércoles 10 de Enero, 2024</t>
-        </is>
-      </c>
-      <c r="I4" s="11" t="inlineStr">
-        <is>
-          <t>Segundo trámite constitucional / Senado — Comparado</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Mensaje</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>C.Diputados</t>
-        </is>
-      </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>15.643-06</t>
+          <t>17.817-07</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 76-374 que retira y hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 122-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -786,27 +786,27 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
+          <t>Constitución, Legislación, Justicia y Reglamento</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>3 de enero de 2023</t>
+          <t>8 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -816,29 +816,29 @@
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>16.888-06</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 69-374 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -853,17 +853,17 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>31 de mayo de 2024</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados — Diario</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -873,64 +873,64 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>16746-06</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Segundo informe de comisión de Medio Ambiente, Cambio Climático y Bienes Nacionales.  COMPARADO DE INDICACIONES</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Abril, 2024</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado — Comparado</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -940,34 +940,34 @@
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>17.797-06</t>
+          <t>16746-06</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
+          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>1 de septiembre de 2025</t>
+          <t>Miércoles 10 de Abril, 2024</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -992,44 +992,44 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno</t>
+          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>17.817-07</t>
+          <t>17.797-06</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
+          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>07/01/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta, oficio N° 282-2025 de la Corte Suprema, por el cual remite opinión respecto del proyecto (informe N° 30-2025).</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1039,12 +1039,12 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Constitución, Legislación, Justicia y Reglamento</t>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>8 de septiembre de 2025</t>
+          <t>1 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Justicia y Derechos Humanos</t>
+          <t>Ministerio Secretaría General de Gobierno</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-06-15
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 111-374 que hace presente la urgencia Suma</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 143-374 que retira y hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -637,47 +637,47 @@
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>15.643-06</t>
+          <t>16.075-06</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 123-374 que retira y hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>3 de enero de 2023</t>
+          <t>4 de julio de 2023</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -692,34 +692,34 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>16.064-06</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 121-374 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -729,59 +729,59 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>3 de julio de 2023</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>17.817-07</t>
+          <t>16.063-06</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
+          <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 122-374 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>Constitución, Legislación, Justicia y Reglamento</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>8 de septiembre de 2025</t>
+          <t>3 de julio de 2023</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -816,29 +816,29 @@
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Justicia y Derechos Humanos</t>
+          <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>16.888-06</t>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 123-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -848,27 +848,27 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>31 de mayo de 2024</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Diario</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -878,91 +878,91 @@
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Segundo informe de comisión de Medio Ambiente, Cambio Climático y Bienes Nacionales.  COMPARADO DE INDICACIONES</t>
+          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 121-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>10 de enero de 2024</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>Segundo trámite constitucional / C.Diputados</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Mensaje</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>Miércoles 10 de Enero, 2024</t>
-        </is>
-      </c>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>Segundo trámite constitucional / Senado — Comparado</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>Mensaje</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>C.Diputados</t>
-        </is>
-      </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>16746-06</t>
+          <t>17.817-07</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
+          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>23/03/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 122-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Constitución, Legislación, Justicia y Reglamento</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Abril, 2024</t>
+          <t>8 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -992,44 +992,44 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
+          <t>Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>17.797-06</t>
+          <t>16.888-06</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
+          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
+          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1039,17 +1039,17 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>1 de septiembre de 2025</t>
+          <t>31 de mayo de 2024</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados — Diario</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
@@ -1064,34 +1064,34 @@
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno</t>
+          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>16.886-12</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Segundo trámite constitucional / Senado — Segundo informe de comisión de Medio Ambiente, Cambio Climático y Bienes Nacionales.  COMPARADO DE INDICACIONES</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1101,59 +1101,59 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>29 de mayo de 2024</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Segundo trámite constitucional / Senado — Comparado</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>17.520-17</t>
+          <t>16746-06</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
+          <t>Modifica la ley N° 20.285, sobre acceso a la informacion pública, para elevar los estándares de transparencia corporativa exigible a las empresas públicas</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>07/05/2025</t>
+          <t>23/03/2026</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 14-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1163,17 +1163,17 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Derechos Humanos y Pueblos Originarios</t>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>5 de mayo de 2025</t>
+          <t>Miércoles 10 de Abril, 2024</t>
         </is>
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -1183,96 +1183,96 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
+          <t>Becker Alvear, Miguel Ángel; Berger Fett, Bernardo; Castro Bascuñán, José Miguel; Fuenzalida Cobo, Juan; Jouannet Valderrama, Andrés; Matheson Villán, Christian; Meza Pereira, José Carlos; Tapia Ramos, Cristián; Weisse Novoa, Flor</t>
         </is>
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>17.446-17</t>
+          <t>17.797-06</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
+          <t>Modifica la ley N° 20.500, sobre Asociaciones y Participación Ciudadana en la Gestión Pública, y otros cuerpos normativos que indica</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>08/04/2025</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 1602-373 que hace presente la urgencia Suma</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Suma</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
+          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>3 de abril de 2025</t>
+          <t>1 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>Isabel Allende Bussi</t>
+          <t>Ministerio Secretaría General de Gobierno</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>16.075-06</t>
+          <t>16.886-12</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
+          <t>Dicta normas sobre protección de personas defensoras de la naturaleza y los derechos humanos medioambientales</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>11/07/2023</t>
+          <t>08/10/2025</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1282,22 +1282,22 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>4 de julio de 2023</t>
+          <t>29 de mayo de 2024</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
@@ -1312,29 +1312,29 @@
       </c>
       <c r="L13" s="12" t="inlineStr">
         <is>
-          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
+          <t>Alejandro Bernales; Viviana Delgado; Luis Malla (A); Vlado Mirosevic; Sebastián Videla</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>16.064-06</t>
+          <t>17.520-17</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
+          <t>Establece la obligación de incorporar la debida diligencia en derechos humanos a las empresas que operen en territorio nacional</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>05/07/2023</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio N° 20406. Deriva a la Comisión de Economía, Fomento; Micro, Pequeña y Mediana Empresa; Protección de los Consumidores y Turismo, el proyecto de ley asignado inicialmente a la Comisión de Derechos Humanos.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1349,17 +1349,17 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Derechos Humanos y Pueblos Originarios</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>3 de julio de 2023</t>
+          <t>5 de mayo de 2025</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1374,29 +1374,29 @@
       </c>
       <c r="L14" s="11" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
+          <t>María Francisca Bello Campos; Roberto Celedón Fernández; Lorena Fries Monleón; Andrés Giordano Salazar; Diego Ibáñez Cotroneo; Camila Rojas Valderrama; Jaime Sáez Quiroz; Clara Sagardia Cabezas; Carolina Tello Rojas; Gael Yeomans Araya</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>16.063-06</t>
+          <t>17.446-17</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
+          <t>Establece y regula la debida diligencia de las empresas en el respeto a los derechos humanos, el medio ambiente y el cambio climático</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>05/07/2023</t>
+          <t>08/04/2025</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta de proyecto . Pasa a Comisión de Gobierno Interior, Nacionalidad, Ciudadanía y Regionalización.</t>
+          <t>Primer trámite constitucional / Senado — Cuenta de proyecto . Pasa a Comisión de Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1406,22 +1406,22 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Gobierno Interior Nacionalidad Ciudadanía y Regionalización</t>
+          <t>Derechos Humanos, Nacionalidad y Ciudadanía</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>3 de julio de 2023</t>
+          <t>3 de abril de 2025</t>
         </is>
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
@@ -1431,12 +1431,12 @@
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
+          <t>Isabel Allende Bussi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-06-22
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>19/06/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 143-374 que retira y hace presente la urgencia Suma</t>
+          <t>Segundo trámite constitucional / Senado — Primer informe de comisión de Hacienda.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Hacienda</t>
+          <t>Cuenta de primer informe de comisión</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Segundo trámite constitucional / Senado — InformeComparado</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-07-06
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>19/06/2026</t>
+          <t>24/06/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Primer informe de comisión de Hacienda.</t>
+          <t>Segundo trámite constitucional / Senado — Discusión general . Aprobado en general Se fija como plazo para presentar indicaciones el 06/07/2026 a las 12:00</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Cuenta de primer informe de comisión</t>
+          <t>Boletín de indicaciones</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — InformeComparado</t>
+          <t>Segundo trámite constitucional / Senado — DiarioVotación</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -637,89 +637,89 @@
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>16.075-06</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>23/06/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 173-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>4 de julio de 2023</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16.064-06</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
+          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 163-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -729,44 +729,44 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>3 de julio de 2023</t>
+          <t>10 de enero de 2024</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Moción</t>
+          <t>Mensaje</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Cámara de Diputados</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>16.063-06</t>
+          <t>16.075-06</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
+          <t>Modifica cuerpos legales que indica en materia de transparencia e información de fondos recibidos por organizaciones de interés público</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>3 de julio de 2023</t>
+          <t>4 de julio de 2023</t>
         </is>
       </c>
       <c r="I5" s="12" t="inlineStr">
@@ -816,54 +816,54 @@
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
+          <t>Danisa Astudillo Peiretti; Miguel Ángel Calisto Águila; Karol Cariola Oliva; Daniella Cicardini Milla; Marcos Ilabaca Cerda; Daniel Manouchehri Lobos; Vlado Mirosevic Verdugo; Javiera Morales Alvarado; Leonardo Soto Ferrada; Renzo Trisotti Martínez</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>15.643-06</t>
+          <t>16.064-06</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
+          <t>Establece una regulación para la conformación y funcionamiento de organizaciones no gubernamentales</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 123-374 que retira y hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Gobierno, Descentralización y Regionalización</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>3 de enero de 2023</t>
+          <t>3 de julio de 2023</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -878,34 +878,34 @@
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
+          <t>Miguel Ángel Calisto Águila; Johannes Kaiser Barents-Von Hohenhagen; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Carolina Tello Rojas</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>16.063-06</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Modifica la ley N° 20.500, sobre asociaciones y participación ciudadana en la gestión pública, para establecer el deber de informar respecto del financiamiento y aportes recibidos de privados</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 121-374 que hace presente la urgencia Simple</t>
+          <t>Primer trámite constitucional / C.Diputados — Archivado. Cuenta oficio N°13/1/2026, de la Comisión de Gobierno Interior, mediante el cual comunica decisión de archivar el proyecto. REMÍTASE AL ARCHIVO</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -915,44 +915,44 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>3 de julio de 2023</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Jorge Brito Hasbún; Andrés Giordano Salazar; Claudia Mix Jiménez; Javiera Morales Alvarado; Ericka Ñanco Vásquez; Maite Orsini Pascal; Camila Rojas Valderrama; Jaime Sáez Quiroz; Consuelo Veloso Ávila</t>
         </is>
       </c>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>17.817-07</t>
+          <t>15.643-06</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
+          <t>Modifica normas legales que indica para obligar a las organizaciones no gubernamentales a transparentar sus ingresos y mecanismos de financiamiento</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 122-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 123-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -972,27 +972,27 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Constitución, Legislación, Justicia y Reglamento</t>
+          <t>Gobierno, Descentralización y Regionalización</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>8 de septiembre de 2025</t>
+          <t>3 de enero de 2023</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Mensaje</t>
+          <t>Moción</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -1002,29 +1002,29 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Justicia y Derechos Humanos</t>
+          <t>Miguel Ángel Calisto Águila; Erika Olivera De La Fuente; Joanna Pérez Olea; Jorge Saffirio Espinoza; Leonardo Soto Ferrada</t>
         </is>
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>16.888-06</t>
+          <t>17.817-07</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
+          <t>Moderniza el régimen normativo de las corporaciones y fundaciones, y fortalece su fiscalización</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
+          <t>Primer trámite constitucional / C.Diputados — Cuenta del Mensaje 122-374 que hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1039,17 +1039,17 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Constitución, Legislación, Justicia y Reglamento</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>31 de mayo de 2024</t>
+          <t>8 de septiembre de 2025</t>
         </is>
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>Primer trámite constitucional / C.Diputados — Diario</t>
+          <t>Primer trámite constitucional / C.Diputados</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
@@ -1064,54 +1064,54 @@
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
+          <t>Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>16.888-06</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Moderniza la regulación del lobby y las gestiones de intereses particulares ante las autoridades y funcionarios</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Segundo informe de comisión de Medio Ambiente, Cambio Climático y Bienes Nacionales.  COMPARADO DE INDICACIONES</t>
+          <t>Primer trámite constitucional / C.Diputados — Discusión general . Queda pendiente</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 10 de Enero, 2024</t>
+          <t>31 de mayo de 2024</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Comparado</t>
+          <t>Primer trámite constitucional / C.Diputados — Diario</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1121,12 +1121,12 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>C.Diputados</t>
+          <t>Cámara de Diputados</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio Secretaría General de Gobierno; Ministerio Secretaría General de la Presidencia; Ministerio de Hacienda; Ministerio de Justicia y Derechos Humanos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-07-20
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,17 +585,17 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>24/06/2026</t>
+          <t>17/07/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Discusión general . Aprobado en general Se fija como plazo para presentar indicaciones el 06/07/2026 a las 12:00</t>
+          <t>Segundo trámite constitucional / Senado — Oficio modificaciones a Cámara de Origen .</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Suma</t>
+          <t>Discusión inmediata</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Boletín de indicaciones</t>
+          <t>Cuenta oficio con modificaciones de Cámara Revisora</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — DiarioVotación</t>
+          <t>Segundo trámite constitucional / Senado — Oficio</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-07-27
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,17 +585,17 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>22/07/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Oficio modificaciones a Cámara de Origen .</t>
+          <t>Disc. informe C.Mixta por rechazo de modif. C. Revisora / Senado — Discusión informe de Comisión Mixta . Queda pendiente Se solicita aplazamiento de la votación.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Discusión inmediata</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Cuenta oficio con modificaciones de Cámara Revisora</t>
+          <t>En Sala</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Oficio</t>
+          <t>Disc. informe C.Mixta por rechazo de modif. C. Revisora / Senado — Diario</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -637,22 +637,22 @@
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>23/06/2026</t>
+          <t>22/07/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 173-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira y formula indicaciones al proyecto. (114-374). Incluye informe financiero complementario N° 170/22.07.2026.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -662,59 +662,59 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>10 de enero de 2024</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>Segundo trámite constitucional / C.Diputados — Oficio</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Mensaje</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>Miércoles 10 de Enero, 2024</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>Segundo trámite constitucional / Senado</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>Mensaje</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>C.Diputados</t>
-        </is>
-      </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>21/07/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 163-374 que hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 215-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -724,22 +724,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -749,12 +749,12 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: actualización semanal 2026-08-03
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,12 +585,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>22/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Disc. informe C.Mixta por rechazo de modif. C. Revisora / Senado — Discusión informe de Comisión Mixta . Queda pendiente Se solicita aplazamiento de la votación.</t>
+          <t>Disc. informe C.Mixta por rechazo de modif. C. Revisora / Senado — Cuenta oficio N° 210-2026 de la Corte Suprema</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Disc. informe C.Mixta por rechazo de modif. C. Revisora / Senado — Diario</t>
+          <t>Disc. informe C.Mixta por rechazo de modif. C. Revisora / Senado — Oficio</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-08-17
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -585,27 +585,27 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>13/08/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Disc. informe C.Mixta por rechazo de modif. C. Revisora / Senado — Cuenta oficio N° 210-2026 de la Corte Suprema</t>
+          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio N° 21499. Comunica al Ejecutivo resultado del veto.</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Discusión inmediata</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>Cámara</t>
         </is>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>En Sala</t>
+          <t>Ingreso fallo del Tribunal Constitucional</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Disc. informe C.Mixta por rechazo de modif. C. Revisora / Senado — Oficio</t>
+          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -647,17 +647,17 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>22/07/2026</t>
+          <t>12/08/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira y formula indicaciones al proyecto. (114-374). Incluye informe financiero complementario N° 170/22.07.2026.</t>
+          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira y formula indicación al proyecto. (137-374). Incluye informe financiero complementario N° 196/12.08.2026.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Simple</t>
+          <t>Sin urgencia</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: actualización semanal 2026-08-24
</commit_message>
<xml_diff>
--- a/seguimiento_legislativo.xlsx
+++ b/seguimiento_legislativo.xlsx
@@ -575,47 +575,47 @@
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>18216-05</t>
+          <t>16553-12</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
+          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>13/08/2026</t>
+          <t>18/08/2026</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio N° 21499. Comunica al Ejecutivo resultado del veto.</t>
+          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 267-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Discusión inmediata</t>
+          <t>Simple</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Cámara</t>
+          <t>Senado</t>
         </is>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Ingreso fallo del Tribunal Constitucional</t>
+          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Miércoles 22 de Abril, 2026</t>
+          <t>Miércoles 10 de Enero, 2024</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Trámite en Tribunal Constitucional / C.Diputados — Oficio</t>
+          <t>Segundo trámite constitucional / Senado</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -630,34 +630,34 @@
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Ministerio de Hacienda</t>
+          <t>Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>16.552-12</t>
+          <t>18216-05</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
+          <t>Para la reconstrucción nacional y el desarrollo económico y social</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>12/08/2026</t>
+          <t>17/08/2026</t>
         </is>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — S.E. el Presidente de la República retira y formula indicación al proyecto. (137-374). Incluye informe financiero complementario N° 196/12.08.2026.</t>
+          <t>Trámite finalización en Cámara de Origen / C.Diputados — Cuenta, Copia autorizada de una resolución del Tribunal Constitucional mediante la cual prorroga por diez días el plazo para resolver el requerimiento de inconstitucionalidad presentado respecto del proyecto.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Sin urgencia</t>
+          <t>Discusión inmediata</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -667,17 +667,17 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+          <t>Oficio resultado veto</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>10 de enero de 2024</t>
+          <t>Miércoles 22 de Abril, 2026</t>
         </is>
       </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / C.Diputados — Oficio</t>
+          <t>Trámite finalización en Cámara de Origen / C.Diputados</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -687,34 +687,34 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Senado</t>
+          <t>C.Diputados</t>
         </is>
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Hacienda</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>16553-12</t>
+          <t>16.552-12</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Fortalece y mejora la eficacia de la fiscalización y el cumplimiento de la regulación ambiental a cargo de la Superintendencia del Medio Ambiente, y regula otras materias que indica</t>
+          <t>Modifica diversos cuerpos legales, con el objeto de fortalecer la institucionalidad ambiental y mejorar su eficiencia</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>21/07/2026</t>
+          <t>17/08/2026</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Segundo trámite constitucional / Senado — Cuenta del Mensaje 215-374 que retira y hace presente la urgencia Simple</t>
+          <t>Segundo trámite constitucional / C.Diputados — Cuenta del Mensaje 262-374 que retira y hace presente la urgencia Simple</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -724,37 +724,37 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Primer informe de comisión Medio Ambiente y Recursos Naturales</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>10 de enero de 2024</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Segundo trámite constitucional / C.Diputados</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Mensaje</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
           <t>Senado</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>Medio Ambiente, Cambio Climático y Bienes Nacionales</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Miércoles 10 de Enero, 2024</t>
-        </is>
-      </c>
-      <c r="I4" s="11" t="inlineStr">
-        <is>
-          <t>Segundo trámite constitucional / Senado</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Mensaje</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>C.Diputados</t>
-        </is>
-      </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Ministerio del Medio Ambiente</t>
+          <t>Ministerio de Agricultura; Ministerio de Economía, Fomento y Turismo; Ministerio de Energía; Ministerio de Hacienda; Ministerio de Obras Públicas; Ministerio del Medio Ambiente</t>
         </is>
       </c>
     </row>

</xml_diff>